<commit_message>
Atualizar insumos e arquivos de avaliacao
</commit_message>
<xml_diff>
--- a/utils/insumos/regra_classificacao.xlsx
+++ b/utils/insumos/regra_classificacao.xlsx
@@ -11,6 +11,9 @@
     <sheet name="regras_classificacao" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="comparadores" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">regras_classificacao!$A$1:$Q$35</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -546,7 +549,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -575,12 +578,6 @@
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -632,16 +629,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -654,7 +655,28 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -840,1488 +862,1490 @@
   <dimension ref="A1:Q35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34.36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="27.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="29.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="51.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34.36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="19.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="33.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="17.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="20.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="55.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="19.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="16.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="29.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="51.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="34.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="33.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="17.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="20.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="55.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="19.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="14.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="79.57"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G2" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H2" s="0" t="n">
+      <c r="E2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="I2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J2" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="K2" s="0" t="s">
+      <c r="J2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="O2" s="0" t="n">
+      <c r="O2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="P2" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q2" s="0" t="s">
+      <c r="P2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q2" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" s="0" t="n">
+      <c r="E3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I3" s="0" t="s">
+      <c r="I3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J3" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="K3" s="0" t="s">
+      <c r="J3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O3" s="0" t="n">
+      <c r="O3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="P3" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q3" s="0" t="s">
+      <c r="P3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q3" s="1" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="0" t="s">
+      <c r="E4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H4" s="0" t="n">
+      <c r="H4" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I4" s="0" t="s">
+      <c r="I4" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J4" s="0" t="s">
+      <c r="J4" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K4" s="0" t="s">
+      <c r="K4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="O4" s="0" t="n">
+      <c r="O4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="P4" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q4" s="0" t="s">
+      <c r="P4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q4" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G5" s="0" t="s">
+      <c r="E5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H5" s="0" t="n">
+      <c r="H5" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I5" s="0" t="s">
+      <c r="I5" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J5" s="0" t="s">
+      <c r="J5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K5" s="0" t="s">
+      <c r="K5" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="O5" s="0" t="n">
+      <c r="O5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="P5" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q5" s="0" t="s">
+      <c r="P5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q5" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G6" s="0" t="s">
+      <c r="E6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="0" t="n">
+      <c r="H6" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I6" s="0" t="s">
+      <c r="I6" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J6" s="0" t="s">
+      <c r="J6" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K6" s="0" t="s">
+      <c r="K6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="O6" s="0" t="n">
+      <c r="O6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="P6" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q6" s="0" t="s">
+      <c r="P6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q6" s="1" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G7" s="0" t="s">
+      <c r="E7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H7" s="0" t="n">
+      <c r="H7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I7" s="0" t="s">
+      <c r="I7" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J7" s="0" t="s">
+      <c r="J7" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K7" s="0" t="s">
+      <c r="K7" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="O7" s="0" t="n">
+      <c r="O7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="P7" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q7" s="0" t="s">
+      <c r="P7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q7" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F8" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G8" s="0" t="s">
+      <c r="E8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H8" s="0" t="n">
+      <c r="H8" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I8" s="0" t="s">
+      <c r="I8" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J8" s="0" t="s">
+      <c r="J8" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K8" s="0" t="s">
+      <c r="K8" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="O8" s="0" t="n">
+      <c r="O8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="P8" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q8" s="0" t="s">
+      <c r="P8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q8" s="1" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G9" s="0" t="s">
+      <c r="E9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H9" s="0" t="n">
+      <c r="H9" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I9" s="0" t="s">
+      <c r="I9" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J9" s="0" t="s">
+      <c r="J9" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K9" s="0" t="s">
+      <c r="K9" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="O9" s="0" t="n">
+      <c r="O9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="P9" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q9" s="0" t="s">
+      <c r="P9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q9" s="1" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G10" s="0" t="s">
+      <c r="E10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H10" s="0" t="n">
+      <c r="H10" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I10" s="0" t="s">
+      <c r="I10" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J10" s="0" t="s">
+      <c r="J10" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K10" s="0" t="s">
+      <c r="K10" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="O10" s="0" t="n">
+      <c r="O10" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="P10" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q10" s="0" t="s">
+      <c r="P10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q10" s="1" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F11" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G11" s="0" t="s">
+      <c r="E11" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H11" s="0" t="n">
+      <c r="H11" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I11" s="0" t="s">
+      <c r="I11" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J11" s="0" t="s">
+      <c r="J11" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K11" s="0" t="s">
+      <c r="K11" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="O11" s="0" t="n">
+      <c r="O11" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="P11" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q11" s="0" t="s">
+      <c r="P11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q11" s="1" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F12" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G12" s="0" t="s">
+      <c r="E12" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H12" s="0" t="n">
+      <c r="H12" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I12" s="0" t="s">
+      <c r="I12" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J12" s="0" t="s">
+      <c r="J12" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K12" s="0" t="s">
+      <c r="K12" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="O12" s="0" t="n">
+      <c r="O12" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="P12" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q12" s="0" t="s">
+      <c r="P12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q12" s="1" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="D13" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F13" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G13" s="0" t="s">
+      <c r="E13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G13" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H13" s="0" t="n">
+      <c r="H13" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I13" s="0" t="s">
+      <c r="I13" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J13" s="0" t="s">
+      <c r="J13" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K13" s="0" t="s">
+      <c r="K13" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="O13" s="0" t="n">
+      <c r="O13" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="P13" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q13" s="0" t="s">
+      <c r="P13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q13" s="1" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="D14" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F14" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G14" s="0" t="s">
+      <c r="E14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H14" s="0" t="n">
+      <c r="H14" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I14" s="0" t="s">
+      <c r="I14" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J14" s="0" t="s">
+      <c r="J14" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K14" s="0" t="s">
+      <c r="K14" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="O14" s="0" t="n">
+      <c r="O14" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="P14" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q14" s="0" t="s">
+      <c r="P14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q14" s="1" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="D15" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F15" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G15" s="0" t="s">
+      <c r="E15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H15" s="0" t="n">
+      <c r="H15" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I15" s="0" t="s">
+      <c r="I15" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J15" s="0" t="s">
+      <c r="J15" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K15" s="0" t="s">
+      <c r="K15" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="O15" s="0" t="n">
+      <c r="O15" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="P15" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q15" s="0" t="s">
+      <c r="P15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q15" s="1" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="D16" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F16" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G16" s="0" t="s">
+      <c r="E16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H16" s="0" t="n">
+      <c r="H16" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I16" s="0" t="s">
+      <c r="I16" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J16" s="0" t="s">
+      <c r="J16" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K16" s="0" t="s">
+      <c r="K16" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="O16" s="0" t="n">
+      <c r="O16" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="P16" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q16" s="0" t="s">
+      <c r="P16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q16" s="1" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="D17" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F17" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G17" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H17" s="0" t="n">
+      <c r="E17" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H17" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I17" s="0" t="s">
+      <c r="I17" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J17" s="0" t="s">
+      <c r="J17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K17" s="0" t="s">
+      <c r="K17" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="O17" s="0" t="n">
+      <c r="O17" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="P17" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q17" s="0" t="s">
+      <c r="P17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q17" s="1" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F18" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G18" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H18" s="0" t="n">
+      <c r="E18" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H18" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="O18" s="0" t="n">
+      <c r="O18" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="P18" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q18" s="0" t="s">
+      <c r="P18" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q18" s="1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="C19" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F19" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G19" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H19" s="0" t="n">
+      <c r="E19" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H19" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="O19" s="0" t="n">
+      <c r="O19" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="P19" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q19" s="0" t="s">
+      <c r="P19" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q19" s="1" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="C20" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F20" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G20" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H20" s="0" t="n">
+      <c r="E20" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H20" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I20" s="0" t="s">
+      <c r="I20" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J20" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="K20" s="0" t="s">
+      <c r="J20" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K20" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O20" s="0" t="n">
+      <c r="O20" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="P20" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q20" s="0" t="s">
+      <c r="P20" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q20" s="1" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="E21" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F21" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G21" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H21" s="0" t="n">
+      <c r="E21" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H21" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I21" s="0" t="s">
+      <c r="I21" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J21" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="K21" s="0" t="s">
+      <c r="J21" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K21" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="O21" s="0" t="n">
-        <v>20</v>
-      </c>
-      <c r="P21" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q21" s="0" t="s">
+      <c r="O21" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="P21" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q21" s="1" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="C22" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D22" s="0" t="s">
+      <c r="D22" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="E22" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F22" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G22" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H22" s="0" t="n">
+      <c r="E22" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H22" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I22" s="0" t="s">
+      <c r="I22" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J22" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="K22" s="0" t="s">
+      <c r="J22" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K22" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="L22" s="0" t="s">
+      <c r="L22" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="M22" s="0" t="s">
+      <c r="M22" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="N22" s="0" t="s">
+      <c r="N22" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="O22" s="0" t="n">
-        <v>21</v>
-      </c>
-      <c r="P22" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q22" s="0" t="s">
+      <c r="O22" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="P22" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q22" s="1" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="C23" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F23" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G23" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H23" s="0" t="n">
+      <c r="E23" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H23" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="I23" s="0" t="s">
+      <c r="I23" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J23" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="K23" s="0" t="s">
+      <c r="J23" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K23" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O23" s="0" t="n">
-        <v>22</v>
-      </c>
-      <c r="P23" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q23" s="0" t="s">
+      <c r="O23" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="P23" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q23" s="1" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="C24" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F24" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G24" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H24" s="0" t="n">
+      <c r="E24" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H24" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="O24" s="0" t="n">
+      <c r="O24" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="P24" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q24" s="0" t="s">
+      <c r="P24" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q24" s="1" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C25" s="0" t="s">
+      <c r="C25" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D25" s="0" t="s">
+      <c r="D25" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="E25" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F25" s="0" t="s">
+      <c r="E25" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G25" s="0" t="s">
+      <c r="G25" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H25" s="0" t="s">
+      <c r="H25" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="O25" s="0" t="n">
+      <c r="O25" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="P25" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q25" s="0" t="s">
+      <c r="P25" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q25" s="1" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="A26" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C26" s="0" t="s">
+      <c r="C26" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D26" s="0" t="s">
+      <c r="D26" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="E26" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F26" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G26" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H26" s="0" t="n">
+      <c r="E26" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H26" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="I26" s="0" t="s">
+      <c r="I26" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J26" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="K26" s="0" t="s">
+      <c r="J26" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K26" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="O26" s="0" t="n">
-        <v>25</v>
-      </c>
-      <c r="P26" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q26" s="0" t="s">
+      <c r="O26" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="P26" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q26" s="1" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="A27" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B27" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C27" s="0" t="s">
+      <c r="C27" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="E27" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F27" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G27" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H27" s="0" t="n">
+      <c r="E27" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H27" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="I27" s="0" t="s">
+      <c r="I27" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J27" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="K27" s="0" t="s">
+      <c r="J27" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K27" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O27" s="0" t="n">
+      <c r="O27" s="1" t="n">
         <v>26</v>
       </c>
-      <c r="P27" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q27" s="0" t="s">
+      <c r="P27" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q27" s="1" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C28" s="0" t="s">
+      <c r="C28" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D28" s="0" t="s">
+      <c r="D28" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="E28" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F28" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G28" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H28" s="0" t="n">
+      <c r="E28" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H28" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="I28" s="0" t="s">
+      <c r="I28" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J28" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="K28" s="0" t="s">
+      <c r="J28" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K28" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="O28" s="0" t="n">
+      <c r="O28" s="1" t="n">
         <v>27</v>
       </c>
-      <c r="P28" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q28" s="0" t="s">
+      <c r="P28" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q28" s="1" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+      <c r="A29" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B29" s="0" t="s">
+      <c r="B29" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="C29" s="0" t="s">
+      <c r="C29" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="E29" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F29" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G29" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H29" s="0" t="n">
+      <c r="E29" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H29" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="I29" s="0" t="s">
+      <c r="I29" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J29" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="K29" s="0" t="s">
+      <c r="J29" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K29" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O29" s="0" t="n">
+      <c r="O29" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="P29" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q29" s="0" t="s">
+      <c r="P29" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q29" s="1" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+      <c r="A30" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B30" s="0" t="s">
+      <c r="B30" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C30" s="0" t="s">
+      <c r="C30" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="E30" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F30" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G30" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H30" s="0" t="n">
+      <c r="E30" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H30" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="I30" s="0" t="s">
+      <c r="I30" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J30" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="K30" s="0" t="s">
+      <c r="J30" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K30" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="O30" s="0" t="n">
+      <c r="O30" s="1" t="n">
         <v>29</v>
       </c>
-      <c r="P30" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q30" s="0" t="s">
+      <c r="P30" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q30" s="1" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="A31" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B31" s="0" t="s">
+      <c r="B31" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C31" s="0" t="s">
+      <c r="C31" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E31" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F31" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G31" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H31" s="0" t="n">
+      <c r="E31" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H31" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="I31" s="0" t="s">
+      <c r="I31" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J31" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="K31" s="0" t="s">
+      <c r="J31" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K31" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O31" s="0" t="n">
+      <c r="O31" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="P31" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q31" s="0" t="s">
+      <c r="P31" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q31" s="1" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+      <c r="A32" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B32" s="0" t="s">
+      <c r="B32" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C32" s="0" t="s">
+      <c r="C32" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F32" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G32" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H32" s="0" t="n">
+      <c r="E32" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H32" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="I32" s="0" t="s">
+      <c r="I32" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J32" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="K32" s="0" t="s">
+      <c r="J32" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K32" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="O32" s="0" t="n">
+      <c r="O32" s="1" t="n">
         <v>31</v>
       </c>
-      <c r="P32" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q32" s="0" t="s">
+      <c r="P32" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q32" s="1" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
+      <c r="A33" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="B33" s="0" t="s">
+      <c r="B33" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C33" s="0" t="s">
+      <c r="C33" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="E33" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F33" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G33" s="0" t="s">
+      <c r="E33" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G33" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="H33" s="0" t="s">
+      <c r="H33" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="I33" s="0" t="s">
+      <c r="I33" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J33" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="K33" s="0" t="s">
+      <c r="J33" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K33" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="O33" s="0" t="n">
+      <c r="O33" s="1" t="n">
         <v>32</v>
       </c>
-      <c r="P33" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q33" s="0" t="s">
+      <c r="P33" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q33" s="1" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
+      <c r="A34" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B34" s="0" t="s">
+      <c r="B34" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="C34" s="0" t="s">
+      <c r="C34" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="E34" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F34" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G34" s="0" t="s">
+      <c r="E34" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G34" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="H34" s="0" t="s">
+      <c r="H34" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="I34" s="0" t="s">
+      <c r="I34" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J34" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="K34" s="0" t="s">
+      <c r="J34" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K34" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O34" s="0" t="n">
+      <c r="O34" s="1" t="n">
         <v>33</v>
       </c>
-      <c r="P34" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q34" s="0" t="s">
+      <c r="P34" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q34" s="1" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+      <c r="A35" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="B35" s="0" t="s">
+      <c r="B35" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="C35" s="0" t="s">
+      <c r="C35" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="E35" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F35" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="G35" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="H35" s="0" t="n">
+      <c r="E35" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H35" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="O35" s="0" t="n">
+      <c r="O35" s="1" t="n">
         <v>34</v>
       </c>
-      <c r="P35" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q35" s="0" t="s">
+      <c r="P35" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q35" s="1" t="s">
         <v>154</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:Q35"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2329,6 +2353,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2340,95 +2365,95 @@
   <dimension ref="A1:B11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="74.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="74.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="0" t="s">
+      <c r="A2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>171</v>
       </c>
     </row>

</xml_diff>